<commit_message>
Lead the summary with the recommendation, not the open PO
The summary sheet listed Amazon's open PO (12,795 units) above the
recommended ship quantity, which reads as though the plan proposes shipping
the whole order book. It does not - it proposes 3,845, or 30% of it.

The summary now leads with SHIP NOW, labels the open PO explicitly as not a
recommendation, and shows the walk from one to the other: less 1,740
unsupplyable, less 7,210 held back to stay inside 35-day cover. Adds an
overstock check giving cover now (29d), after this shipment (43d), and if
the full open PO were shipped (77d), plus the 1,472 units of inherited
excess sitting in SKUs this plan ships nothing to.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N5QckZ42nw4ueLobVZghMn
</commit_message>
<xml_diff>
--- a/analysis/cocoblu-supply-2026-09-04/Cocoblu_Supply_Plan_v5_ISK3.xlsx
+++ b/analysis/cocoblu-supply-2026-09-04/Cocoblu_Supply_Plan_v5_ISK3.xlsx
@@ -17,7 +17,7 @@
     <sheet name="7_EOL - cancel these" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'0_Summary'!$A$1:$B$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'0_Summary'!$A$1:$B$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1_Dispatch by PO'!$A$1:$F$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2_Dispatch lines'!$A$1:$N$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3_SKU plan 35d'!$A$1:$S$105</definedName>
@@ -445,10 +445,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -467,53 +467,35 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Scope</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Vendor code QZ73J / FC ISK3 only</t>
-        </is>
+          <t>&gt;&gt;&gt; RECOMMENDED SHIP NOW (units)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3845</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cover policy</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>35d cap on ESTABLISHED SKUs only</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>New arrivals</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>No cap - ship Amazon full ask (no DRR to cap on)</t>
-        </is>
-      </c>
-    </row>
+          <t>&gt;&gt;&gt; Recommended ship value (INR, vendor cost)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>6833367</v>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sellable inventory at Cocoblu (3 Sep)</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>7815</v>
+          <t>-- how we get there --</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Open PO in scope (7 POs, ASN = 0)</t>
+          <t>Amazon open PO in scope (NOT a recommendation)</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -523,135 +505,255 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>RECOMMENDED SHIP NOW (units)</t>
+          <t xml:space="preserve">  less: unsupplyable (EOL or out of stock)</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3845</v>
+        <v>-1740</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Recommended ship value (INR, vendor cost)</t>
+          <t xml:space="preserve">  less: held back - would breach 35d cover</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6833367</v>
+        <v>-7210</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Hold / cancel (units)</t>
+          <t xml:space="preserve">  = SHIP NOW</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8950</v>
+        <v>3845</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Units needed with no PO cover (ask Amazon)</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>604</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>SKUs shipped</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>29</v>
-      </c>
-    </row>
+          <t xml:space="preserve">  ship as % of open PO</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Max DOH - established SKUs after ship</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>36</t>
+          <t>-- overstock check --</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>New arrival units (group A - new PO)</t>
+          <t>Established SKUs shipped</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1200</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>New arrival units (group B - never sold)</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>168</v>
+          <t>Max DOH of any established SKU after ship</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Excluded - no supply</t>
+          <t>Account cover now (days)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Click 20000, Quad Pro 1.5m 60W, Zeno 65W retractable</t>
+          <t>29</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Excluded - EOL (no Tally sale FY26-27)</t>
+          <t>Account cover after this shipment (days)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>6 SKUs / 177u / Rs 156,034</t>
+          <t>43</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Excluded - other vendor code</t>
+          <t>Account cover IF we shipped the full open PO</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PPAFS / 147u at HBA4, HKA2, HNR4, HPN6</t>
+          <t>77</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>Inherited excess above 35d we ship nothing to</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1472</v>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>-- scope &amp; policy --</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Vendor code QZ73J / FC ISK3 only</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Cover policy</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>35d cap on ESTABLISHED SKUs only</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>New arrivals</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>No cap - ship full ask (no DRR to cap on)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Sellable inventory at Cocoblu (3 Sep)</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>7815</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Units needed with no PO cover (ask Amazon)</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>New arrival units (group A - new PO)</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>New arrival units (group B - never sold)</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Excluded - no supply</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Click 20000, Quad Pro 1.5m 60W, Zeno 65W retractable</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Excluded - EOL (no Tally sale FY26-27)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>6 SKUs / 177u</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Excluded - other vendor code</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>PPAFS / 147u at HBA4, HKA2, HNR4, HPN6</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>Excluded - EXPIRED PO</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>39VRVKCF / 1,105u - window closed 1 Sep, get it cancelled</t>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>39VRVKCF / 1,105u - window closed 1 Sep</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B18"/>
+  <autoFilter ref="A1:B31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>